<commit_message>
Batch update to conform with the latest CEDAR model
</commit_message>
<xml_diff>
--- a/10x-multiome/latest/10x-multiome.xlsx
+++ b/10x-multiome/latest/10x-multiome.xlsx
@@ -35,10 +35,10 @@
     </comment>
     <comment ref="B1" authorId="1">
       <text>
-        <t>A locally assigned identifier provided by the data provider for the dataset. It
-is used to reference an external metadata record that may be maintained
-independently, enabling traceability and supporting provenance tracking.
-Example: Visium_9OLC_A4_S1</t>
+        <t>An identifier assigned by the data provider to reference an external metadata
+record for the dataset. The external record may be maintained independently and
+can support dataset traceability and provenance tracking. Leave this field empty
+if no such identifier exists.</t>
       </text>
     </comment>
     <comment ref="C1" authorId="1">
@@ -129,7 +129,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="236">
   <si>
     <t>parent_sample_id</t>
   </si>
@@ -143,304 +143,364 @@
     <t>dataset_type</t>
   </si>
   <si>
+    <t>Cell DIVE</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000159</t>
+  </si>
+  <si>
+    <t>CODEX</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000160</t>
+  </si>
+  <si>
+    <t>Light Sheet</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000168</t>
+  </si>
+  <si>
+    <t>MIBI</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000172</t>
+  </si>
+  <si>
+    <t>LC-MS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000194</t>
+  </si>
+  <si>
     <t>HiFi-Slide</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000195</t>
   </si>
   <si>
+    <t>Histology</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000197</t>
+  </si>
+  <si>
+    <t>PhenoCycler</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000199</t>
+  </si>
+  <si>
+    <t>CyCIF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000200</t>
+  </si>
+  <si>
+    <t>MALDI</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000201</t>
+  </si>
+  <si>
+    <t>SIMS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000202</t>
+  </si>
+  <si>
+    <t>DESI</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000204</t>
+  </si>
+  <si>
+    <t>Auto-fluorescence</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000205</t>
+  </si>
+  <si>
+    <t>Confocal</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000206</t>
+  </si>
+  <si>
+    <t>Thick section Multiphoton MxIF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000207</t>
+  </si>
+  <si>
+    <t>Second Harmonic Generation (SHG)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000208</t>
+  </si>
+  <si>
+    <t>Enhanced Stimulated Raman Spectroscopy (SRS)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000209</t>
+  </si>
+  <si>
+    <t>10X Multiome</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000215</t>
+  </si>
+  <si>
+    <t>Molecular Cartography</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000217</t>
+  </si>
+  <si>
+    <t>CosMx Transcriptomics</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000218</t>
+  </si>
+  <si>
+    <t>Xenium</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000219</t>
+  </si>
+  <si>
+    <t>MERFISH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000221</t>
+  </si>
+  <si>
     <t>SNARE-seq2</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000264</t>
   </si>
   <si>
+    <t>2D Imaging Mass Cytometry</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000296</t>
+  </si>
+  <si>
+    <t>GeoMx (NGS)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000300</t>
+  </si>
+  <si>
+    <t>GeoMx (nCounter)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000301</t>
+  </si>
+  <si>
+    <t>Visium (no probes)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000302</t>
+  </si>
+  <si>
+    <t>Visium (with probes)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000303</t>
+  </si>
+  <si>
+    <t>ATACseq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000309</t>
+  </si>
+  <si>
+    <t>RNAseq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000310</t>
+  </si>
+  <si>
+    <t>RNAseq (with probes)</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000311</t>
+  </si>
+  <si>
+    <t>nanoSPLITS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000312</t>
+  </si>
+  <si>
+    <t>MUSIC</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000328</t>
+  </si>
+  <si>
+    <t>Resolve</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000384</t>
+  </si>
+  <si>
+    <t>Stereo-seq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000385</t>
+  </si>
+  <si>
+    <t>Seq-Scope</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000390</t>
+  </si>
+  <si>
+    <t>DART-FISH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000396</t>
+  </si>
+  <si>
+    <t>seqFISH</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000397</t>
+  </si>
+  <si>
+    <t>MS Lipidomics</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000405</t>
+  </si>
+  <si>
+    <t>CyTOF</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000407</t>
+  </si>
+  <si>
+    <t>DBiT-seq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000428</t>
+  </si>
+  <si>
+    <t>Singular Genomics G4X</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000429</t>
+  </si>
+  <si>
+    <t>CosMx Proteomics</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000435</t>
+  </si>
+  <si>
+    <t>FACS</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000440</t>
+  </si>
+  <si>
+    <t>Olink</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000441</t>
+  </si>
+  <si>
+    <t>4i</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000447</t>
+  </si>
+  <si>
+    <t>MPLEx</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000448</t>
+  </si>
+  <si>
+    <t>Pixel-seqV2</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000450</t>
+  </si>
+  <si>
+    <t>Visium HD</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000451</t>
+  </si>
+  <si>
     <t>COMET</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000458</t>
   </si>
   <si>
-    <t>Visium (no probes)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000302</t>
-  </si>
-  <si>
-    <t>DESI</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000204</t>
-  </si>
-  <si>
-    <t>Confocal</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000206</t>
-  </si>
-  <si>
-    <t>Stereo-seq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000385</t>
-  </si>
-  <si>
-    <t>Visium (with probes)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000303</t>
-  </si>
-  <si>
-    <t>Molecular Cartography</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000217</t>
-  </si>
-  <si>
-    <t>DBiT-seq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000428</t>
-  </si>
-  <si>
-    <t>Seq-Scope</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000390</t>
-  </si>
-  <si>
-    <t>CosMx Transcriptomics</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000218</t>
-  </si>
-  <si>
-    <t>CyCIF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000200</t>
-  </si>
-  <si>
-    <t>Light Sheet</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000168</t>
-  </si>
-  <si>
-    <t>seqFISH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000397</t>
-  </si>
-  <si>
-    <t>ATACseq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000309</t>
-  </si>
-  <si>
-    <t>CosMx Proteomics</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000435</t>
-  </si>
-  <si>
-    <t>Singular Genomics G4X</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000429</t>
-  </si>
-  <si>
-    <t>Visium HD</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000451</t>
-  </si>
-  <si>
-    <t>MERFISH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000221</t>
-  </si>
-  <si>
-    <t>10X Multiome</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000215</t>
-  </si>
-  <si>
-    <t>4i</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000447</t>
-  </si>
-  <si>
-    <t>PhenoCycler</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000199</t>
-  </si>
-  <si>
-    <t>Second Harmonic Generation (SHG)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000208</t>
-  </si>
-  <si>
-    <t>Thick section Multiphoton MxIF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000207</t>
-  </si>
-  <si>
-    <t>CyTOF</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000407</t>
-  </si>
-  <si>
-    <t>Olink</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000441</t>
-  </si>
-  <si>
-    <t>MIBI</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000172</t>
-  </si>
-  <si>
-    <t>Auto-fluorescence</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000205</t>
-  </si>
-  <si>
-    <t>FACS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000440</t>
-  </si>
-  <si>
-    <t>Xenium</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000219</t>
-  </si>
-  <si>
-    <t>SIMS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000202</t>
-  </si>
-  <si>
-    <t>Cell DIVE</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000159</t>
-  </si>
-  <si>
-    <t>CODEX</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000160</t>
-  </si>
-  <si>
-    <t>GeoMx (NGS)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000300</t>
-  </si>
-  <si>
-    <t>MUSIC</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000328</t>
-  </si>
-  <si>
-    <t>Pixel-seqV2</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000450</t>
-  </si>
-  <si>
-    <t>MALDI</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000201</t>
-  </si>
-  <si>
-    <t>2D Imaging Mass Cytometry</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000296</t>
-  </si>
-  <si>
-    <t>Histology</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000197</t>
-  </si>
-  <si>
-    <t>Enhanced Stimulated Raman Spectroscopy (SRS)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000209</t>
-  </si>
-  <si>
-    <t>DART-FISH</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000396</t>
-  </si>
-  <si>
-    <t>Resolve</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000384</t>
-  </si>
-  <si>
-    <t>RNAseq</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000310</t>
-  </si>
-  <si>
-    <t>LC-MS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000194</t>
-  </si>
-  <si>
-    <t>nanoSPLITS</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000312</t>
-  </si>
-  <si>
-    <t>GeoMx (nCounter)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000301</t>
-  </si>
-  <si>
-    <t>RNAseq (with probes)</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000311</t>
-  </si>
-  <si>
-    <t>MS Lipidomics</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000405</t>
-  </si>
-  <si>
-    <t>MPLEx</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000448</t>
+    <t>Virtual Histology</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000473</t>
+  </si>
+  <si>
+    <t>Raman Imaging</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000475</t>
+  </si>
+  <si>
+    <t>STARmap</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000476</t>
+  </si>
+  <si>
+    <t>iCLAP</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000479</t>
+  </si>
+  <si>
+    <t>MACSima</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000480</t>
+  </si>
+  <si>
+    <t>Illumina Spatial ver0</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000487</t>
+  </si>
+  <si>
+    <t>DNA Methylation</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000490</t>
+  </si>
+  <si>
+    <t>Paired-Tag</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000492</t>
+  </si>
+  <si>
+    <t>snm3C-seq</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000504</t>
+  </si>
+  <si>
+    <t>Whole Exome Sequencing</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000514</t>
   </si>
   <si>
     <t>contributors_path</t>
@@ -461,22 +521,58 @@
     <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C126386</t>
   </si>
   <si>
+    <t>Not applicable</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
+  </si>
+  <si>
+    <t>Thermo Fisher Scientific</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_008452</t>
+  </si>
+  <si>
+    <t>Hamamatsu</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_017105</t>
+  </si>
+  <si>
     <t>Leica Biosystems</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_023603</t>
   </si>
   <si>
-    <t>Not applicable</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C48660</t>
-  </si>
-  <si>
-    <t>Thermo Fisher Scientific</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_008452</t>
+    <t>Ionpath</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023605</t>
+  </si>
+  <si>
+    <t>10x Genomics</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023672</t>
+  </si>
+  <si>
+    <t>HTX Technologies</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023734</t>
+  </si>
+  <si>
+    <t>Akoya Biosciences</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023774</t>
+  </si>
+  <si>
+    <t>SunChrom</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023908</t>
   </si>
   <si>
     <t>Roche Diagnostics</t>
@@ -485,43 +581,97 @@
     <t>https://identifiers.org/RRID:SCR_025096</t>
   </si>
   <si>
-    <t>HTX Technologies</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023734</t>
-  </si>
-  <si>
-    <t>10x Genomics</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023672</t>
-  </si>
-  <si>
-    <t>Hamamatsu</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_017105</t>
-  </si>
-  <si>
-    <t>SunChrom</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023908</t>
-  </si>
-  <si>
     <t>preparation_instrument_model</t>
   </si>
   <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
+  </si>
+  <si>
+    <t>Chromium Controller</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_019326</t>
+  </si>
+  <si>
+    <t>Sublimator</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023729</t>
+  </si>
+  <si>
+    <t>M3+ Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023731</t>
+  </si>
+  <si>
+    <t>TM-Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023732</t>
+  </si>
+  <si>
+    <t>M5 Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023733</t>
+  </si>
+  <si>
     <t>NanoZoomer S210</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_023760</t>
   </si>
   <si>
-    <t>Sublimator</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023729</t>
+    <t>NanoZoomer S360</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023761</t>
+  </si>
+  <si>
+    <t>NanoZoomer S60</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023762</t>
+  </si>
+  <si>
+    <t>SunCollect Sprayer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023907</t>
+  </si>
+  <si>
+    <t>AutoStainer XL</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_023957</t>
+  </si>
+  <si>
+    <t>Chromium iX</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024536</t>
+  </si>
+  <si>
+    <t>Chromium X</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024537</t>
+  </si>
+  <si>
+    <t>Visium CytAssist</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_024570</t>
+  </si>
+  <si>
+    <t>ST5020 Multistainer</t>
+  </si>
+  <si>
+    <t>https://identifiers.org/RRID:SCR_025021</t>
   </si>
   <si>
     <t>EVOS M7000</t>
@@ -530,109 +680,91 @@
     <t>https://identifiers.org/RRID:SCR_025070</t>
   </si>
   <si>
-    <t>Chromium Controller</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_019326</t>
-  </si>
-  <si>
-    <t>NanoZoomer S360</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023761</t>
-  </si>
-  <si>
-    <t>NanoZoomer S60</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023762</t>
-  </si>
-  <si>
-    <t>Chromium X</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024537</t>
-  </si>
-  <si>
-    <t>AutoStainer XL</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023957</t>
-  </si>
-  <si>
-    <t>Visium CytAssist</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024570</t>
-  </si>
-  <si>
-    <t>SunCollect Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023907</t>
-  </si>
-  <si>
-    <t>M3+ Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023731</t>
-  </si>
-  <si>
     <t>Discovery Ultra</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_025097</t>
   </si>
   <si>
-    <t>ST5020 Multistainer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_025021</t>
-  </si>
-  <si>
-    <t>Chromium iX</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_024536</t>
-  </si>
-  <si>
     <t>Chromium Connect</t>
   </si>
   <si>
     <t>https://identifiers.org/RRID:SCR_025146</t>
   </si>
   <si>
-    <t>M5 Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023733</t>
-  </si>
-  <si>
-    <t>TM-Sprayer</t>
-  </si>
-  <si>
-    <t>https://identifiers.org/RRID:SCR_023732</t>
-  </si>
-  <si>
     <t>preparation_instrument_kit</t>
   </si>
   <si>
+    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 16 rxn; PN 1000283</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000250</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 4 rxn; PN 1000285</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000251</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Chip J Single Cell Kit, 48 rxns; PN 1000234</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000262</t>
+  </si>
+  <si>
+    <t>10x Genomics; Chromium Next GEM Chip J Single Cell Kit, 16 rxns; PN 1000230</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000263</t>
+  </si>
+  <si>
+    <t>10X Genomics; Visium FFPE Reagent Kit v2-Small, PN 1000436</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000324</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip Q Single Cell Kit, 16 rxns; PN 1000422</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000325</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 48 rxns; PN 1000286</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000367</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 16 rxns; PN 1000287</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000368</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip K Automated Single Cell Kit, 48 rxns; PN 1000289</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000373</t>
+  </si>
+  <si>
+    <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 48 rxns; PN 1000120</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000378</t>
+  </si>
+  <si>
     <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 16 rxns; PN 1000127</t>
   </si>
   <si>
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000379</t>
   </si>
   <si>
-    <t>10X Genomics; Chromium Next GEM Chip K Automated Single Cell Kit, 48 rxns; PN 1000289</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000373</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 16 rxn; PN 1000283</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000250</t>
+    <t>10x Genomics; Chromium GEM-X Single Cell 3' Kit v4, 16 rxns; PN 1000691</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000400</t>
   </si>
   <si>
     <t>10x Genomics; Chromium Single Cell B Chip Kit, 16 rxns; PN 1000074</t>
@@ -641,52 +773,40 @@
     <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000462</t>
   </si>
   <si>
-    <t>10X Genomics; Chromium NextGem Single Cell Multiome ATAC + Gene Expression Reagent Bundle, 4 rxn; PN 1000285</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000251</t>
-  </si>
-  <si>
-    <t>10x Genomics; Chromium GEM-X Single Cell 3' Kit v4, 16 rxns; PN 1000691</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000400</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 48 rxns; PN 1000286</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000367</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip G Single Cell Kit, 48 rxns; PN 1000120</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000378</t>
-  </si>
-  <si>
-    <t>10X Genomics; Visium FFPE Reagent Kit v2-Small, PN 1000436</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000324</t>
-  </si>
-  <si>
-    <t>Custom</t>
-  </si>
-  <si>
-    <t>http://ncicb.nci.nih.gov/xml/owl/EVS/Thesaurus.owl#C65167</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip Q Single Cell Kit, 16 rxns; PN 1000422</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000325</t>
-  </si>
-  <si>
-    <t>10X Genomics; Chromium Next GEM Chip K Single Cell Kit, 16 rxns; PN 1000287</t>
-  </si>
-  <si>
-    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000368</t>
+    <t>10x Genomics; Chromium Chip E Single Cell ATAC Kit, 48 rxns; PN 1000155</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000470</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Human Transcriptome, 6.5 mm, 4 runs; PN 1000675</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000493</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Mouse Transcriptome, 6.5 mm, 4 runs; PN 1000676</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000494</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Human Transcriptome, 11 mm, 4 runs; PN 1001037</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000495</t>
+  </si>
+  <si>
+    <t>10x Genomics; Visium HD, Mouse Transcriptome, 11 mm, 4 runs; PN 1001038</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000496</t>
+  </si>
+  <si>
+    <t>10x Genomics; GEM-X Flex Gene Expression Chip Kit, 4 chips; PN 1000791</t>
+  </si>
+  <si>
+    <t>https://purl.humanatlas.io/vocab/hravs#HRAVS_0000498</t>
   </si>
   <si>
     <t>number_of_pre_amplification_pcr_cycles</t>
@@ -710,7 +830,7 @@
     <t>pav:createdOn</t>
   </si>
   <si>
-    <t>2025-10-21T13:32:33-07:00</t>
+    <t>2026-10-21T13:36:23-07:00</t>
   </si>
   <si>
     <t>pav:derivedFrom</t>
@@ -827,51 +947,51 @@
         <v>3</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="F1" t="s" s="1">
-        <v>105</v>
+        <v>125</v>
       </c>
       <c r="G1" t="s" s="1">
-        <v>106</v>
+        <v>126</v>
       </c>
       <c r="H1" t="s" s="1">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="I1" t="s" s="1">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="J1" t="s" s="1">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="K1" t="s" s="1">
-        <v>186</v>
+        <v>226</v>
       </c>
       <c r="L1" t="s" s="1">
-        <v>187</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2">
       <c r="D2" t="s" s="5">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="L2" t="s" s="13">
-        <v>188</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="5">
     <dataValidation type="list" sqref="D2:D1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'dataset_type'!$A$1:$A$50</formula1>
+      <formula1>'dataset_type'!$A$1:$A$60</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="H2:H1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_instrument_vendor'!$A$1:$A$9</formula1>
+      <formula1>'preparation_instrument_vendor'!$A$1:$A$11</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="I2:I1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_instrument_model'!$A$1:$A$18</formula1>
+      <formula1>'preparation_instrument_model'!$A$1:$A$19</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="J2:J1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="" showErrorMessage="true">
-      <formula1>'preparation_instrument_kit'!$A$1:$A$12</formula1>
+      <formula1>'preparation_instrument_kit'!$A$1:$A$20</formula1>
     </dataValidation>
     <dataValidation type="whole" operator="between" sqref="K2:K1001" allowBlank="true" errorStyle="stop" errorTitle="Validation Error" error="Value should be a number" showErrorMessage="true">
       <formula1>-2147483648</formula1>
@@ -886,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B60"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1287,6 +1407,86 @@
       </c>
       <c r="B50" t="s" s="0">
         <v>103</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>104</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>110</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>112</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1296,79 +1496,95 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>108</v>
+        <v>128</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>109</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>111</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>113</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>114</v>
+        <v>134</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>115</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>117</v>
+        <v>137</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>119</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>121</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>122</v>
+        <v>142</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>123</v>
+        <v>143</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>124</v>
+        <v>144</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>125</v>
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>146</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>148</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -1378,151 +1594,159 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>112</v>
+        <v>151</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>113</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>129</v>
+        <v>153</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>130</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>131</v>
+        <v>155</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>132</v>
+        <v>156</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>134</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>135</v>
+        <v>159</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>136</v>
+        <v>160</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>137</v>
+        <v>161</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>138</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>139</v>
+        <v>163</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>140</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>141</v>
+        <v>165</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>142</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>143</v>
+        <v>167</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>144</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>145</v>
+        <v>169</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>146</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>147</v>
+        <v>171</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>148</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>149</v>
+        <v>173</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>150</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>151</v>
+        <v>175</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>152</v>
+        <v>176</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>153</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>154</v>
+        <v>178</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>155</v>
+        <v>179</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>156</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>157</v>
+        <v>181</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>158</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>159</v>
+        <v>183</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>160</v>
+        <v>184</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>185</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -1532,103 +1756,167 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>163</v>
+        <v>152</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>165</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>166</v>
+        <v>190</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>167</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>168</v>
+        <v>192</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>169</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>170</v>
+        <v>194</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>171</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>172</v>
+        <v>196</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>173</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>174</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>175</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>176</v>
+        <v>200</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>177</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>178</v>
+        <v>202</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>179</v>
+        <v>203</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>180</v>
+        <v>204</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>181</v>
+        <v>205</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>182</v>
+        <v>206</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>183</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>184</v>
+        <v>208</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>185</v>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>212</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>214</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>216</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>218</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>220</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>222</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>224</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>225</v>
       </c>
     </row>
   </sheetData>
@@ -1649,30 +1937,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>189</v>
+        <v>229</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>190</v>
+        <v>230</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>192</v>
+        <v>232</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>194</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>191</v>
+        <v>231</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>193</v>
+        <v>233</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>195</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>